<commit_message>
Fixed chronological date sorting in queries, restored full asset detail view, and finalized 34-point HTBasic preflight
</commit_message>
<xml_diff>
--- a/Template_DCV_Reference_732A.xlsx
+++ b/Template_DCV_Reference_732A.xlsx
@@ -1,28 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ziyanang\PycharmProjects\WelcomeScreen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A42BAA-8B4B-408F-B424-A1911A184AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C617DE9-6EB1-4557-8195-A607F39FE4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3615000" sheetId="1" r:id="rId1"/>
     <sheet name="5009002" sheetId="2" r:id="rId2"/>
     <sheet name="4621005" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="83">
   <si>
     <t>Category</t>
   </si>
@@ -39,9 +52,6 @@
     <t>Serial Number</t>
   </si>
   <si>
-    <t>3615000</t>
-  </si>
-  <si>
     <t>Equipment ID</t>
   </si>
   <si>
@@ -51,187 +61,229 @@
     <t>Set ID</t>
   </si>
   <si>
+    <t>Note: Tracks 10V and 1V outputs. Uncertainty is in nV.</t>
+  </si>
+  <si>
+    <t>Date (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>10V Measured (V)</t>
+  </si>
+  <si>
+    <t>10V Uncert (nV)</t>
+  </si>
+  <si>
+    <t>1V Measured (V)</t>
+  </si>
+  <si>
+    <t>1V Uncert (nV)</t>
+  </si>
+  <si>
+    <t>Facility Location</t>
+  </si>
+  <si>
+    <t>Pressure (hPa)</t>
+  </si>
+  <si>
+    <t>Cert Number</t>
+  </si>
+  <si>
+    <t>Reviewer Comment</t>
+  </si>
+  <si>
+    <t>2019-10-07</t>
+  </si>
+  <si>
+    <t>Loveland</t>
+  </si>
+  <si>
+    <t>1-11582565623-1</t>
+  </si>
+  <si>
+    <t>2020-05-28</t>
+  </si>
+  <si>
+    <t>1-12646956191-1</t>
+  </si>
+  <si>
+    <t>2021-02-03</t>
+  </si>
+  <si>
+    <t>1-13640405443-1</t>
+  </si>
+  <si>
+    <t>2021-09-02</t>
+  </si>
+  <si>
+    <t>1-15055696422-1</t>
+  </si>
+  <si>
+    <t>2022-04-08</t>
+  </si>
+  <si>
+    <t>Roseville</t>
+  </si>
+  <si>
+    <t>1-16849189133-1</t>
+  </si>
+  <si>
+    <t>2023-03-03</t>
+  </si>
+  <si>
+    <t>WO-00371279</t>
+  </si>
+  <si>
+    <t>2024-05-14</t>
+  </si>
+  <si>
+    <t>WO-00679822</t>
+  </si>
+  <si>
+    <t>2025-05-01</t>
+  </si>
+  <si>
+    <t>WO-01037969</t>
+  </si>
+  <si>
+    <t>2026-05-19</t>
+  </si>
+  <si>
+    <t>WO-01394837</t>
+  </si>
+  <si>
+    <t>732C</t>
+  </si>
+  <si>
+    <t>5009002</t>
+  </si>
+  <si>
+    <t>PN010075</t>
+  </si>
+  <si>
+    <t>Set 1</t>
+  </si>
+  <si>
+    <t>1-13640053356-1</t>
+  </si>
+  <si>
+    <t>2022-03-21</t>
+  </si>
+  <si>
+    <t>1-16555467063-1</t>
+  </si>
+  <si>
+    <t>2022-11-07</t>
+  </si>
+  <si>
+    <t>WO-00275556</t>
+  </si>
+  <si>
+    <t>2023-08-29</t>
+  </si>
+  <si>
+    <t>WO-00469028</t>
+  </si>
+  <si>
+    <t>2024-08-23</t>
+  </si>
+  <si>
+    <t>WO-00770555</t>
+  </si>
+  <si>
+    <t>2025-11-14</t>
+  </si>
+  <si>
+    <t>WO-01127666</t>
+  </si>
+  <si>
+    <t>4621005</t>
+  </si>
+  <si>
+    <t>PC4732</t>
+  </si>
+  <si>
+    <t>Set 3</t>
+  </si>
+  <si>
+    <t>2020-01-26</t>
+  </si>
+  <si>
+    <t>1-12191838135-1</t>
+  </si>
+  <si>
+    <t>2021-02-05</t>
+  </si>
+  <si>
+    <t>1-13901257728-1</t>
+  </si>
+  <si>
+    <t>2022-02-14</t>
+  </si>
+  <si>
+    <t>1-16277333536-1</t>
+  </si>
+  <si>
+    <t>2023-03-21</t>
+  </si>
+  <si>
+    <t>WO-00402648</t>
+  </si>
+  <si>
+    <t>2024-12-18</t>
+  </si>
+  <si>
+    <t>WO-00924716</t>
+  </si>
+  <si>
+    <t>2026-03-20</t>
+  </si>
+  <si>
+    <t>WO-01312271</t>
+  </si>
+  <si>
+    <t>DCVoltageReference</t>
+  </si>
+  <si>
+    <t>SerialNumber</t>
+  </si>
+  <si>
+    <t>EquipmentID</t>
+  </si>
+  <si>
+    <t>SetID</t>
+  </si>
+  <si>
+    <t>Note:Tracks10Vand1Voutputs.UncertaintyisinnV.</t>
+  </si>
+  <si>
+    <t>Date(YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>10VMeasured(V)</t>
+  </si>
+  <si>
+    <t>10VUncert(nV)</t>
+  </si>
+  <si>
+    <t>1VMeasured(V)</t>
+  </si>
+  <si>
+    <t>1VUncert(nV)</t>
+  </si>
+  <si>
+    <t>FacilityLocation</t>
+  </si>
+  <si>
+    <t>Pressure(hPa)</t>
+  </si>
+  <si>
+    <t>CertNumber</t>
+  </si>
+  <si>
+    <t>ReviewerComment</t>
+  </si>
+  <si>
     <t>Set 2</t>
-  </si>
-  <si>
-    <t>Note: Tracks 10V and 1V outputs. Uncertainty is in nV.</t>
-  </si>
-  <si>
-    <t>Date (YYYY-MM-DD)</t>
-  </si>
-  <si>
-    <t>10V Measured (V)</t>
-  </si>
-  <si>
-    <t>10V Uncert (nV)</t>
-  </si>
-  <si>
-    <t>1V Measured (V)</t>
-  </si>
-  <si>
-    <t>1V Uncert (nV)</t>
-  </si>
-  <si>
-    <t>Facility Location</t>
-  </si>
-  <si>
-    <t>Pressure (hPa)</t>
-  </si>
-  <si>
-    <t>Cert Number</t>
-  </si>
-  <si>
-    <t>Reviewer Comment</t>
-  </si>
-  <si>
-    <t>2019-10-07</t>
-  </si>
-  <si>
-    <t>Loveland</t>
-  </si>
-  <si>
-    <t>1-11582565623-1</t>
-  </si>
-  <si>
-    <t>2020-05-28</t>
-  </si>
-  <si>
-    <t>1-12646956191-1</t>
-  </si>
-  <si>
-    <t>2021-02-03</t>
-  </si>
-  <si>
-    <t>1-13640405443-1</t>
-  </si>
-  <si>
-    <t>2021-09-02</t>
-  </si>
-  <si>
-    <t>1-15055696422-1</t>
-  </si>
-  <si>
-    <t>2022-04-08</t>
-  </si>
-  <si>
-    <t>Roseville</t>
-  </si>
-  <si>
-    <t>1-16849189133-1</t>
-  </si>
-  <si>
-    <t>2023-03-03</t>
-  </si>
-  <si>
-    <t>WO-00371279</t>
-  </si>
-  <si>
-    <t>2024-05-14</t>
-  </si>
-  <si>
-    <t>WO-00679822</t>
-  </si>
-  <si>
-    <t>2025-05-01</t>
-  </si>
-  <si>
-    <t>WO-01037969</t>
-  </si>
-  <si>
-    <t>2026-05-19</t>
-  </si>
-  <si>
-    <t>WO-01394837</t>
-  </si>
-  <si>
-    <t>732C</t>
-  </si>
-  <si>
-    <t>5009002</t>
-  </si>
-  <si>
-    <t>PN010075</t>
-  </si>
-  <si>
-    <t>Set 1</t>
-  </si>
-  <si>
-    <t>1-13640053356-1</t>
-  </si>
-  <si>
-    <t>2022-03-21</t>
-  </si>
-  <si>
-    <t>1-16555467063-1</t>
-  </si>
-  <si>
-    <t>2022-11-07</t>
-  </si>
-  <si>
-    <t>WO-00275556</t>
-  </si>
-  <si>
-    <t>2023-08-29</t>
-  </si>
-  <si>
-    <t>WO-00469028</t>
-  </si>
-  <si>
-    <t>2024-08-23</t>
-  </si>
-  <si>
-    <t>WO-00770555</t>
-  </si>
-  <si>
-    <t>2025-11-14</t>
-  </si>
-  <si>
-    <t>WO-01127666</t>
-  </si>
-  <si>
-    <t>4621005</t>
-  </si>
-  <si>
-    <t>PC4732</t>
-  </si>
-  <si>
-    <t>Set 3</t>
-  </si>
-  <si>
-    <t>2020-01-26</t>
-  </si>
-  <si>
-    <t>1-12191838135-1</t>
-  </si>
-  <si>
-    <t>2021-02-05</t>
-  </si>
-  <si>
-    <t>1-13901257728-1</t>
-  </si>
-  <si>
-    <t>2022-02-14</t>
-  </si>
-  <si>
-    <t>1-16277333536-1</t>
-  </si>
-  <si>
-    <t>2023-03-21</t>
-  </si>
-  <si>
-    <t>WO-00402648</t>
-  </si>
-  <si>
-    <t>2024-12-18</t>
-  </si>
-  <si>
-    <t>WO-00924716</t>
-  </si>
-  <si>
-    <t>2026-03-20</t>
-  </si>
-  <si>
-    <t>WO-01312271</t>
   </si>
 </sst>
 </file>
@@ -315,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -326,6 +378,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,8 +685,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -641,15 +698,15 @@
     <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -657,67 +714,67 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="B3" s="10">
+        <v>3615000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>17</v>
+        <v>79</v>
       </c>
       <c r="H7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="B8" s="6">
         <v>10.0000713618</v>
@@ -725,22 +782,26 @@
       <c r="C8" s="7">
         <v>161</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="D8" s="5">
+        <v>0.99998895700000001</v>
+      </c>
+      <c r="E8" s="7">
+        <v>42</v>
+      </c>
       <c r="F8" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G8" s="5">
         <v>847</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B9" s="6">
         <v>10.000070789</v>
@@ -748,22 +809,26 @@
       <c r="C9" s="7">
         <v>161</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="D9" s="5">
+        <v>0.99998801999999998</v>
+      </c>
+      <c r="E9" s="7">
+        <v>42</v>
+      </c>
       <c r="F9" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G9" s="5">
         <v>843</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B10" s="6">
         <v>10.000069995</v>
@@ -771,22 +836,26 @@
       <c r="C10" s="7">
         <v>65</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="D10" s="5">
+        <v>0.999986924</v>
+      </c>
+      <c r="E10" s="7">
+        <v>42</v>
+      </c>
       <c r="F10" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G10" s="5">
         <v>847</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="6">
         <v>10.000070733999999</v>
@@ -794,22 +863,26 @@
       <c r="C11" s="7">
         <v>65</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="5">
+        <v>0.99998646472727259</v>
+      </c>
+      <c r="E11" s="7">
+        <v>42</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G11" s="5">
         <v>845</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B12" s="6">
         <v>10.000072931</v>
@@ -817,22 +890,26 @@
       <c r="C12" s="7">
         <v>65</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="D12" s="5">
+        <v>0.99998530550000009</v>
+      </c>
+      <c r="E12" s="7">
+        <v>42</v>
+      </c>
       <c r="F12" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G12" s="5">
         <v>1013</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B13" s="6">
         <v>10.000073799000001</v>
@@ -840,22 +917,26 @@
       <c r="C13" s="7">
         <v>35</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="D13" s="5">
+        <v>0.99998409899999996</v>
+      </c>
+      <c r="E13" s="7">
+        <v>23</v>
+      </c>
       <c r="F13" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G13" s="5">
         <v>1011</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B14" s="6">
         <v>10.000074421000001</v>
@@ -863,20 +944,26 @@
       <c r="C14" s="7">
         <v>34</v>
       </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="D14" s="5">
+        <v>0.99998296600000003</v>
+      </c>
+      <c r="E14" s="7">
+        <v>26</v>
+      </c>
       <c r="F14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14" s="5"/>
+        <v>28</v>
+      </c>
+      <c r="G14" s="5">
+        <v>1013</v>
+      </c>
       <c r="H14" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I14" s="5"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B15" s="6">
         <v>10.000079439</v>
@@ -884,20 +971,26 @@
       <c r="C15" s="7">
         <v>36</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="D15" s="5">
+        <v>0.999981974</v>
+      </c>
+      <c r="E15" s="7">
+        <v>26</v>
+      </c>
       <c r="F15" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G15" s="5"/>
+        <v>28</v>
+      </c>
+      <c r="G15" s="5">
+        <v>1008</v>
+      </c>
       <c r="H15" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I15" s="5"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B16" s="6">
         <v>10.000083883</v>
@@ -905,18 +998,25 @@
       <c r="C16" s="7">
         <v>35</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="D16" s="5">
+        <v>0.99998243799999997</v>
+      </c>
+      <c r="E16" s="7">
+        <v>24.4</v>
+      </c>
       <c r="F16" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G16" s="5">
         <v>1013</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I16" s="5"/>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E27" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -926,7 +1026,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -938,7 +1038,7 @@
     <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -946,75 +1046,75 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="I7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" s="6">
         <v>10.000069359999999</v>
@@ -1022,22 +1122,26 @@
       <c r="C8" s="7">
         <v>121</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="D8" s="5">
+        <v>1.0000941350000001</v>
+      </c>
+      <c r="E8" s="7">
+        <v>82</v>
+      </c>
       <c r="F8" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G8" s="5">
         <v>847</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B9" s="6">
         <v>10.000057183999999</v>
@@ -1045,22 +1149,26 @@
       <c r="C9" s="7">
         <v>121</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="D9">
+        <v>1.0000917659999999</v>
+      </c>
+      <c r="E9" s="7">
+        <v>82</v>
+      </c>
       <c r="F9" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G9" s="5">
         <v>1017</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B10" s="6">
         <v>10.000053983000001</v>
@@ -1068,22 +1176,26 @@
       <c r="C10" s="7">
         <v>121</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="D10" s="5">
+        <v>1.0000936090000001</v>
+      </c>
+      <c r="E10" s="7">
+        <v>29</v>
+      </c>
       <c r="F10" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G10" s="5">
         <v>1006</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B11" s="6">
         <v>10.000048175</v>
@@ -1091,22 +1203,26 @@
       <c r="C11" s="7">
         <v>25</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="5">
+        <v>1.0000936380000001</v>
+      </c>
+      <c r="E11" s="7">
+        <v>27</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G11" s="5">
         <v>1006</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B12" s="6">
         <v>10.000044315</v>
@@ -1114,22 +1230,26 @@
       <c r="C12" s="7">
         <v>24</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="D12" s="5">
+        <v>1.000094525</v>
+      </c>
+      <c r="E12" s="7">
+        <v>27</v>
+      </c>
       <c r="F12" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G12" s="5">
         <v>1010</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B13" s="6">
         <v>10.00004055</v>
@@ -1137,16 +1257,20 @@
       <c r="C13" s="7">
         <v>27</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="D13" s="5">
+        <v>1.0000919749999999</v>
+      </c>
+      <c r="E13" s="7">
+        <v>27</v>
+      </c>
       <c r="F13" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G13" s="5">
         <v>1010</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I13" s="5"/>
     </row>
@@ -1158,7 +1282,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1170,7 +1294,7 @@
     <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1178,75 +1302,75 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="B8" s="6">
         <v>10.000027867</v>
@@ -1254,22 +1378,26 @@
       <c r="C8" s="7">
         <v>111</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="D8" s="5">
+        <v>1.0000616847999999</v>
+      </c>
+      <c r="E8" s="7">
+        <v>95</v>
+      </c>
       <c r="F8" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G8" s="5">
         <v>845</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B9" s="6">
         <v>10.000016567999999</v>
@@ -1277,22 +1405,26 @@
       <c r="C9" s="7">
         <v>121</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="D9" s="5">
+        <v>1.000060771</v>
+      </c>
+      <c r="E9" s="9">
+        <v>82</v>
+      </c>
       <c r="F9" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G9" s="5">
         <v>844</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B10" s="6">
         <v>10.000013897000001</v>
@@ -1300,22 +1432,26 @@
       <c r="C10" s="7">
         <v>121</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="D10" s="6">
+        <v>1.00060543</v>
+      </c>
+      <c r="E10" s="7">
+        <v>82</v>
+      </c>
       <c r="F10" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G10" s="5">
         <v>1006</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B11" s="6">
         <v>10.000010205000001</v>
@@ -1323,22 +1459,26 @@
       <c r="C11" s="7">
         <v>24</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="5">
+        <v>1.000059757</v>
+      </c>
+      <c r="E11" s="7">
+        <v>25</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G11" s="5">
         <v>1010</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B12" s="6">
         <v>10.000003099000001</v>
@@ -1346,22 +1486,26 @@
       <c r="C12" s="7">
         <v>27</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="D12" s="5">
+        <v>1.000058296</v>
+      </c>
+      <c r="E12" s="7">
+        <v>28</v>
+      </c>
       <c r="F12" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G12" s="5">
         <v>1016</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B13" s="6">
         <v>10.000000035999999</v>
@@ -1369,16 +1513,20 @@
       <c r="C13" s="7">
         <v>30</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="D13" s="5">
+        <v>1.0000060356</v>
+      </c>
+      <c r="E13" s="7">
+        <v>30</v>
+      </c>
       <c r="F13" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G13" s="5">
         <v>1013</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13" s="5"/>
     </row>

</xml_diff>